<commit_message>
Username and Passwords change
</commit_message>
<xml_diff>
--- a/Customers.xlsx
+++ b/Customers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/myrysbaev/Documents/Websites/makro-route/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E40F609-10DF-2B48-9612-DF783D12610C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8228A5ED-EFFD-054E-BA15-8B1EE8D4E260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34200" yWindow="600" windowWidth="51200" windowHeight="28200" xr2:uid="{52332BE9-A126-CC46-B047-61E72F4E335D}"/>
   </bookViews>
@@ -2110,9 +2110,6 @@
     <t>Andalucia Mediterranean grocery</t>
   </si>
   <si>
-    <t>Morton Road</t>
-  </si>
-  <si>
     <t>77493</t>
   </si>
   <si>
@@ -3408,6 +3405,9 @@
   </si>
   <si>
     <t>8821 Westheimer Road #109</t>
+  </si>
+  <si>
+    <t>20140 Morton Road</t>
   </si>
 </sst>
 </file>
@@ -3814,7 +3814,7 @@
         <v>673</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="C2" t="s">
         <v>25</v>
@@ -3871,22 +3871,22 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
+        <v>934</v>
+      </c>
+      <c r="B5" t="s">
         <v>935</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>1109</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
         <v>936</v>
-      </c>
-      <c r="C5" t="s">
-        <v>1110</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" t="s">
-        <v>937</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.15">
@@ -3931,10 +3931,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A8" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="B8" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="C8" t="s">
         <v>48</v>
@@ -3946,7 +3946,7 @@
         <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.15">
@@ -4014,7 +4014,7 @@
         <v>675</v>
       </c>
       <c r="B12" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="C12" t="s">
         <v>676</v>
@@ -4134,7 +4134,7 @@
         <v>546</v>
       </c>
       <c r="B18" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="C18" t="s">
         <v>545</v>
@@ -4271,13 +4271,13 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A25" t="s">
+        <v>876</v>
+      </c>
+      <c r="B25" t="s">
         <v>877</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>878</v>
-      </c>
-      <c r="C25" t="s">
-        <v>879</v>
       </c>
       <c r="D25" t="s">
         <v>49</v>
@@ -4286,7 +4286,7 @@
         <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.15">
@@ -4346,7 +4346,7 @@
         <v>10</v>
       </c>
       <c r="F28" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.15">
@@ -4391,22 +4391,22 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A31" t="s">
+        <v>974</v>
+      </c>
+      <c r="B31" t="s">
         <v>975</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
+        <v>939</v>
+      </c>
+      <c r="D31" t="s">
+        <v>17</v>
+      </c>
+      <c r="E31" t="s">
+        <v>10</v>
+      </c>
+      <c r="F31" t="s">
         <v>976</v>
-      </c>
-      <c r="C31" t="s">
-        <v>940</v>
-      </c>
-      <c r="D31" t="s">
-        <v>17</v>
-      </c>
-      <c r="E31" t="s">
-        <v>10</v>
-      </c>
-      <c r="F31" t="s">
-        <v>977</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.15">
@@ -4437,7 +4437,7 @@
         <v>36</v>
       </c>
       <c r="C33" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="D33" t="s">
         <v>17</v>
@@ -4571,22 +4571,22 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A40" t="s">
+        <v>937</v>
+      </c>
+      <c r="B40" t="s">
         <v>938</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>939</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
+        <v>17</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" t="s">
         <v>940</v>
-      </c>
-      <c r="D40" t="s">
-        <v>17</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F40" t="s">
-        <v>941</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.15">
@@ -4613,8 +4613,8 @@
       <c r="A42" t="s">
         <v>688</v>
       </c>
-      <c r="B42" t="s">
-        <v>689</v>
+      <c r="B42" s="1" t="s">
+        <v>1121</v>
       </c>
       <c r="C42" t="s">
         <v>558</v>
@@ -4626,7 +4626,7 @@
         <v>10</v>
       </c>
       <c r="F42" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.15">
@@ -4731,10 +4731,10 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A48" t="s">
+        <v>854</v>
+      </c>
+      <c r="B48" t="s">
         <v>855</v>
-      </c>
-      <c r="B48" t="s">
-        <v>856</v>
       </c>
       <c r="C48" t="s">
         <v>57</v>
@@ -4771,10 +4771,10 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A50" t="s">
+        <v>690</v>
+      </c>
+      <c r="B50" t="s">
         <v>691</v>
-      </c>
-      <c r="B50" t="s">
-        <v>692</v>
       </c>
       <c r="C50" t="s">
         <v>25</v>
@@ -4934,10 +4934,10 @@
         <v>210</v>
       </c>
       <c r="B58" t="s">
+        <v>1091</v>
+      </c>
+      <c r="C58" t="s">
         <v>1092</v>
-      </c>
-      <c r="C58" t="s">
-        <v>1093</v>
       </c>
       <c r="D58" t="s">
         <v>17</v>
@@ -5031,10 +5031,10 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A63" t="s">
+        <v>692</v>
+      </c>
+      <c r="B63" t="s">
         <v>693</v>
-      </c>
-      <c r="B63" t="s">
-        <v>694</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>25</v>
@@ -5046,27 +5046,27 @@
         <v>10</v>
       </c>
       <c r="F63" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A64" t="s">
+        <v>941</v>
+      </c>
+      <c r="B64" t="s">
         <v>942</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
+        <v>939</v>
+      </c>
+      <c r="D64" t="s">
+        <v>17</v>
+      </c>
+      <c r="E64" t="s">
+        <v>10</v>
+      </c>
+      <c r="F64" t="s">
         <v>943</v>
-      </c>
-      <c r="C64" t="s">
-        <v>940</v>
-      </c>
-      <c r="D64" t="s">
-        <v>17</v>
-      </c>
-      <c r="E64" t="s">
-        <v>10</v>
-      </c>
-      <c r="F64" t="s">
-        <v>944</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.15">
@@ -5151,22 +5151,22 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A69" t="s">
+        <v>695</v>
+      </c>
+      <c r="B69" t="s">
         <v>696</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C69" t="s">
         <v>697</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
+        <v>17</v>
+      </c>
+      <c r="E69" t="s">
+        <v>10</v>
+      </c>
+      <c r="F69" t="s">
         <v>698</v>
-      </c>
-      <c r="D69" t="s">
-        <v>17</v>
-      </c>
-      <c r="E69" t="s">
-        <v>10</v>
-      </c>
-      <c r="F69" t="s">
-        <v>699</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.15">
@@ -5191,10 +5191,10 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A71" t="s">
+        <v>699</v>
+      </c>
+      <c r="B71" t="s">
         <v>700</v>
-      </c>
-      <c r="B71" t="s">
-        <v>701</v>
       </c>
       <c r="C71" t="s">
         <v>25</v>
@@ -5211,13 +5211,13 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A72" t="s">
+        <v>985</v>
+      </c>
+      <c r="B72" t="s">
         <v>986</v>
       </c>
-      <c r="B72" t="s">
-        <v>987</v>
-      </c>
       <c r="C72" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="D72" t="s">
         <v>17</v>
@@ -5226,7 +5226,7 @@
         <v>10</v>
       </c>
       <c r="F72" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.15">
@@ -5251,30 +5251,30 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A74" t="s">
+        <v>705</v>
+      </c>
+      <c r="B74" t="s">
         <v>706</v>
       </c>
-      <c r="B74" t="s">
+      <c r="C74" t="s">
         <v>707</v>
       </c>
-      <c r="C74" t="s">
+      <c r="D74" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E74" t="s">
+        <v>10</v>
+      </c>
+      <c r="F74" t="s">
         <v>708</v>
-      </c>
-      <c r="D74" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E74" t="s">
-        <v>10</v>
-      </c>
-      <c r="F74" t="s">
-        <v>709</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A75" t="s">
+        <v>703</v>
+      </c>
+      <c r="B75" t="s">
         <v>704</v>
-      </c>
-      <c r="B75" t="s">
-        <v>705</v>
       </c>
       <c r="C75" t="s">
         <v>565</v>
@@ -5291,10 +5291,10 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A76" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="B76" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C76" t="s">
         <v>552</v>
@@ -5306,15 +5306,15 @@
         <v>10</v>
       </c>
       <c r="F76" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A77" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="B77" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="C77" t="s">
         <v>180</v>
@@ -5331,10 +5331,10 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A78" t="s">
+        <v>710</v>
+      </c>
+      <c r="B78" t="s">
         <v>711</v>
-      </c>
-      <c r="B78" t="s">
-        <v>712</v>
       </c>
       <c r="C78" t="s">
         <v>158</v>
@@ -5346,15 +5346,15 @@
         <v>10</v>
       </c>
       <c r="F78" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A79" t="s">
+        <v>712</v>
+      </c>
+      <c r="B79" t="s">
         <v>713</v>
-      </c>
-      <c r="B79" t="s">
-        <v>714</v>
       </c>
       <c r="C79" t="s">
         <v>25</v>
@@ -5371,10 +5371,10 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A80" t="s">
+        <v>716</v>
+      </c>
+      <c r="B80" t="s">
         <v>717</v>
-      </c>
-      <c r="B80" t="s">
-        <v>718</v>
       </c>
       <c r="C80" t="s">
         <v>25</v>
@@ -5386,38 +5386,38 @@
         <v>10</v>
       </c>
       <c r="F80" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A81" t="s">
+        <v>944</v>
+      </c>
+      <c r="B81" t="s">
         <v>945</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C81" t="s">
+        <v>1090</v>
+      </c>
+      <c r="D81" t="s">
+        <v>17</v>
+      </c>
+      <c r="E81" t="s">
+        <v>10</v>
+      </c>
+      <c r="F81" t="s">
         <v>946</v>
-      </c>
-      <c r="C81" t="s">
-        <v>1091</v>
-      </c>
-      <c r="D81" t="s">
-        <v>17</v>
-      </c>
-      <c r="E81" t="s">
-        <v>10</v>
-      </c>
-      <c r="F81" t="s">
-        <v>947</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A82" t="s">
+        <v>983</v>
+      </c>
+      <c r="B82" t="s">
         <v>984</v>
       </c>
-      <c r="B82" t="s">
-        <v>985</v>
-      </c>
       <c r="C82" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="D82" t="s">
         <v>17</v>
@@ -5426,7 +5426,7 @@
         <v>10</v>
       </c>
       <c r="F82" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.15">
@@ -5491,22 +5491,22 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A86" t="s">
+        <v>719</v>
+      </c>
+      <c r="B86" t="s">
         <v>720</v>
       </c>
-      <c r="B86" t="s">
+      <c r="C86" t="s">
         <v>721</v>
       </c>
-      <c r="C86" t="s">
+      <c r="D86" t="s">
+        <v>17</v>
+      </c>
+      <c r="E86" t="s">
+        <v>10</v>
+      </c>
+      <c r="F86" t="s">
         <v>722</v>
-      </c>
-      <c r="D86" t="s">
-        <v>17</v>
-      </c>
-      <c r="E86" t="s">
-        <v>10</v>
-      </c>
-      <c r="F86" t="s">
-        <v>723</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.15">
@@ -5591,22 +5591,22 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A91" t="s">
+        <v>947</v>
+      </c>
+      <c r="B91" t="s">
         <v>948</v>
       </c>
-      <c r="B91" t="s">
+      <c r="C91" t="s">
+        <v>939</v>
+      </c>
+      <c r="D91" t="s">
+        <v>17</v>
+      </c>
+      <c r="E91" t="s">
+        <v>10</v>
+      </c>
+      <c r="F91" t="s">
         <v>949</v>
-      </c>
-      <c r="C91" t="s">
-        <v>940</v>
-      </c>
-      <c r="D91" t="s">
-        <v>17</v>
-      </c>
-      <c r="E91" t="s">
-        <v>10</v>
-      </c>
-      <c r="F91" t="s">
-        <v>950</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.15">
@@ -5711,10 +5711,10 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A97" t="s">
+        <v>950</v>
+      </c>
+      <c r="B97" t="s">
         <v>951</v>
-      </c>
-      <c r="B97" t="s">
-        <v>952</v>
       </c>
       <c r="C97" t="s">
         <v>63</v>
@@ -5726,7 +5726,7 @@
         <v>10</v>
       </c>
       <c r="F97" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.15">
@@ -5734,7 +5734,7 @@
         <v>114</v>
       </c>
       <c r="B98" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="C98" t="s">
         <v>115</v>
@@ -5771,10 +5771,10 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A100" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B100" t="s">
         <v>1030</v>
-      </c>
-      <c r="B100" t="s">
-        <v>1031</v>
       </c>
       <c r="C100" t="s">
         <v>63</v>
@@ -5791,22 +5791,22 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A101" t="s">
+        <v>953</v>
+      </c>
+      <c r="B101" t="s">
         <v>954</v>
       </c>
-      <c r="B101" t="s">
+      <c r="C101" t="s">
+        <v>939</v>
+      </c>
+      <c r="D101" t="s">
+        <v>17</v>
+      </c>
+      <c r="E101" t="s">
+        <v>10</v>
+      </c>
+      <c r="F101" t="s">
         <v>955</v>
-      </c>
-      <c r="C101" t="s">
-        <v>940</v>
-      </c>
-      <c r="D101" t="s">
-        <v>17</v>
-      </c>
-      <c r="E101" t="s">
-        <v>10</v>
-      </c>
-      <c r="F101" t="s">
-        <v>956</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.15">
@@ -5817,7 +5817,7 @@
         <v>250</v>
       </c>
       <c r="C102" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="D102" t="s">
         <v>17</v>
@@ -5874,7 +5874,7 @@
         <v>59</v>
       </c>
       <c r="B105" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="C105" t="s">
         <v>57</v>
@@ -5891,10 +5891,10 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A106" t="s">
+        <v>723</v>
+      </c>
+      <c r="B106" t="s">
         <v>724</v>
-      </c>
-      <c r="B106" t="s">
-        <v>725</v>
       </c>
       <c r="C106" t="s">
         <v>25</v>
@@ -6077,10 +6077,10 @@
         <v>139</v>
       </c>
       <c r="C115" t="s">
+        <v>1071</v>
+      </c>
+      <c r="D115" t="s">
         <v>1072</v>
-      </c>
-      <c r="D115" t="s">
-        <v>1073</v>
       </c>
       <c r="E115" t="s">
         <v>10</v>
@@ -6097,7 +6097,7 @@
         <v>142</v>
       </c>
       <c r="C116" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="D116" t="s">
         <v>17</v>
@@ -6117,7 +6117,7 @@
         <v>583</v>
       </c>
       <c r="C117" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="D117" t="s">
         <v>17</v>
@@ -6314,7 +6314,7 @@
         <v>284</v>
       </c>
       <c r="B127" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="C127" t="s">
         <v>285</v>
@@ -6351,7 +6351,7 @@
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A129" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B129" t="s">
         <v>674</v>
@@ -6374,7 +6374,7 @@
         <v>585</v>
       </c>
       <c r="B130" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="C130" t="s">
         <v>25</v>
@@ -6411,22 +6411,22 @@
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A132" t="s">
+        <v>977</v>
+      </c>
+      <c r="B132" t="s">
         <v>978</v>
       </c>
-      <c r="B132" t="s">
+      <c r="C132" t="s">
+        <v>939</v>
+      </c>
+      <c r="D132" t="s">
+        <v>17</v>
+      </c>
+      <c r="E132" t="s">
+        <v>10</v>
+      </c>
+      <c r="F132" t="s">
         <v>979</v>
-      </c>
-      <c r="C132" t="s">
-        <v>940</v>
-      </c>
-      <c r="D132" t="s">
-        <v>17</v>
-      </c>
-      <c r="E132" t="s">
-        <v>10</v>
-      </c>
-      <c r="F132" t="s">
-        <v>980</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.15">
@@ -6434,7 +6434,7 @@
         <v>287</v>
       </c>
       <c r="B133" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="C133" t="s">
         <v>489</v>
@@ -6454,7 +6454,7 @@
         <v>289</v>
       </c>
       <c r="B134" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="C134" t="s">
         <v>290</v>
@@ -6474,7 +6474,7 @@
         <v>292</v>
       </c>
       <c r="B135" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="C135" t="s">
         <v>150</v>
@@ -6491,10 +6491,10 @@
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A136" t="s">
+        <v>726</v>
+      </c>
+      <c r="B136" t="s">
         <v>727</v>
-      </c>
-      <c r="B136" t="s">
-        <v>728</v>
       </c>
       <c r="C136" t="s">
         <v>25</v>
@@ -6506,7 +6506,7 @@
         <v>10</v>
       </c>
       <c r="F136" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.15">
@@ -6631,10 +6631,10 @@
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A143" t="s">
+        <v>729</v>
+      </c>
+      <c r="B143" t="s">
         <v>730</v>
-      </c>
-      <c r="B143" t="s">
-        <v>731</v>
       </c>
       <c r="C143" t="s">
         <v>545</v>
@@ -6646,7 +6646,7 @@
         <v>10</v>
       </c>
       <c r="F143" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.15">
@@ -6731,10 +6731,10 @@
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A148" t="s">
+        <v>732</v>
+      </c>
+      <c r="B148" t="s">
         <v>733</v>
-      </c>
-      <c r="B148" t="s">
-        <v>734</v>
       </c>
       <c r="C148" t="s">
         <v>552</v>
@@ -6746,7 +6746,7 @@
         <v>10</v>
       </c>
       <c r="F148" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.15">
@@ -6771,10 +6771,10 @@
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A150" t="s">
+        <v>735</v>
+      </c>
+      <c r="B150" t="s">
         <v>736</v>
-      </c>
-      <c r="B150" t="s">
-        <v>737</v>
       </c>
       <c r="C150" t="s">
         <v>25</v>
@@ -6791,10 +6791,10 @@
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A151" t="s">
+        <v>737</v>
+      </c>
+      <c r="B151" t="s">
         <v>738</v>
-      </c>
-      <c r="B151" t="s">
-        <v>739</v>
       </c>
       <c r="C151" t="s">
         <v>25</v>
@@ -6811,10 +6811,10 @@
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A152" t="s">
+        <v>739</v>
+      </c>
+      <c r="B152" t="s">
         <v>740</v>
-      </c>
-      <c r="B152" t="s">
-        <v>741</v>
       </c>
       <c r="C152" t="s">
         <v>25</v>
@@ -6831,10 +6831,10 @@
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A153" t="s">
+        <v>741</v>
+      </c>
+      <c r="B153" t="s">
         <v>742</v>
-      </c>
-      <c r="B153" t="s">
-        <v>743</v>
       </c>
       <c r="C153" t="s">
         <v>558</v>
@@ -6851,10 +6851,10 @@
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A154" t="s">
+        <v>746</v>
+      </c>
+      <c r="B154" t="s">
         <v>747</v>
-      </c>
-      <c r="B154" t="s">
-        <v>748</v>
       </c>
       <c r="C154" t="s">
         <v>25</v>
@@ -6866,15 +6866,15 @@
         <v>10</v>
       </c>
       <c r="F154" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A155" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="B155" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="C155" t="s">
         <v>25</v>
@@ -6891,10 +6891,10 @@
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A156" t="s">
+        <v>749</v>
+      </c>
+      <c r="B156" t="s">
         <v>750</v>
-      </c>
-      <c r="B156" t="s">
-        <v>751</v>
       </c>
       <c r="C156" t="s">
         <v>540</v>
@@ -6911,10 +6911,10 @@
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A157" t="s">
+        <v>744</v>
+      </c>
+      <c r="B157" t="s">
         <v>745</v>
-      </c>
-      <c r="B157" t="s">
-        <v>746</v>
       </c>
       <c r="C157" t="s">
         <v>25</v>
@@ -6974,7 +6974,7 @@
         <v>314</v>
       </c>
       <c r="B160" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="C160" t="s">
         <v>315</v>
@@ -7137,7 +7137,7 @@
         <v>320</v>
       </c>
       <c r="C168" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="D168" t="s">
         <v>17</v>
@@ -7211,10 +7211,10 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A172" t="s">
+        <v>751</v>
+      </c>
+      <c r="B172" t="s">
         <v>752</v>
-      </c>
-      <c r="B172" t="s">
-        <v>753</v>
       </c>
       <c r="C172" t="s">
         <v>25</v>
@@ -7231,10 +7231,10 @@
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A173" t="s">
+        <v>753</v>
+      </c>
+      <c r="B173" t="s">
         <v>754</v>
-      </c>
-      <c r="B173" t="s">
-        <v>755</v>
       </c>
       <c r="C173" t="s">
         <v>25</v>
@@ -7246,7 +7246,7 @@
         <v>10</v>
       </c>
       <c r="F173" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.15">
@@ -7277,7 +7277,7 @@
         <v>533</v>
       </c>
       <c r="C175" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="D175" t="s">
         <v>17</v>
@@ -7491,13 +7491,13 @@
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A186" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="B186" t="s">
         <v>346</v>
       </c>
       <c r="C186" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="D186" t="s">
         <v>17</v>
@@ -7571,10 +7571,10 @@
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A190" t="s">
+        <v>756</v>
+      </c>
+      <c r="B190" t="s">
         <v>757</v>
-      </c>
-      <c r="B190" t="s">
-        <v>758</v>
       </c>
       <c r="C190" t="s">
         <v>540</v>
@@ -7734,7 +7734,7 @@
         <v>356</v>
       </c>
       <c r="B198" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="C198" t="s">
         <v>180</v>
@@ -7791,10 +7791,10 @@
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A201" t="s">
+        <v>758</v>
+      </c>
+      <c r="B201" t="s">
         <v>759</v>
-      </c>
-      <c r="B201" t="s">
-        <v>760</v>
       </c>
       <c r="C201" t="s">
         <v>152</v>
@@ -7811,10 +7811,10 @@
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A202" t="s">
+        <v>839</v>
+      </c>
+      <c r="B202" t="s">
         <v>840</v>
-      </c>
-      <c r="B202" t="s">
-        <v>841</v>
       </c>
       <c r="C202" t="s">
         <v>25</v>
@@ -7831,22 +7831,22 @@
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A203" t="s">
+        <v>841</v>
+      </c>
+      <c r="B203" t="s">
         <v>842</v>
       </c>
-      <c r="B203" t="s">
+      <c r="C203" t="s">
+        <v>1084</v>
+      </c>
+      <c r="D203" t="s">
+        <v>17</v>
+      </c>
+      <c r="E203" t="s">
+        <v>10</v>
+      </c>
+      <c r="F203" t="s">
         <v>843</v>
-      </c>
-      <c r="C203" t="s">
-        <v>1085</v>
-      </c>
-      <c r="D203" t="s">
-        <v>17</v>
-      </c>
-      <c r="E203" t="s">
-        <v>10</v>
-      </c>
-      <c r="F203" t="s">
-        <v>844</v>
       </c>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.15">
@@ -7871,10 +7871,10 @@
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A205" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B205" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="C205" t="s">
         <v>25</v>
@@ -7886,15 +7886,15 @@
         <v>10</v>
       </c>
       <c r="F205" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A206" t="s">
+        <v>846</v>
+      </c>
+      <c r="B206" t="s">
         <v>847</v>
-      </c>
-      <c r="B206" t="s">
-        <v>848</v>
       </c>
       <c r="C206" t="s">
         <v>111</v>
@@ -7906,27 +7906,27 @@
         <v>10</v>
       </c>
       <c r="F206" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A207" t="s">
+        <v>849</v>
+      </c>
+      <c r="B207" t="s">
         <v>850</v>
       </c>
-      <c r="B207" t="s">
+      <c r="C207" t="s">
         <v>851</v>
       </c>
-      <c r="C207" t="s">
+      <c r="D207" t="s">
         <v>852</v>
       </c>
-      <c r="D207" t="s">
+      <c r="E207" t="s">
+        <v>10</v>
+      </c>
+      <c r="F207" t="s">
         <v>853</v>
-      </c>
-      <c r="E207" t="s">
-        <v>10</v>
-      </c>
-      <c r="F207" t="s">
-        <v>854</v>
       </c>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.15">
@@ -8051,7 +8051,7 @@
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A214" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B214" t="s">
         <v>90</v>
@@ -8191,10 +8191,10 @@
     </row>
     <row r="221" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A221" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B221" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="C221" t="s">
         <v>158</v>
@@ -8206,7 +8206,7 @@
         <v>10</v>
       </c>
       <c r="F221" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="222" spans="1:6" x14ac:dyDescent="0.15">
@@ -8217,7 +8217,7 @@
         <v>386</v>
       </c>
       <c r="C222" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="D222" t="s">
         <v>17</v>
@@ -8231,22 +8231,22 @@
     </row>
     <row r="223" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A223" t="s">
+        <v>858</v>
+      </c>
+      <c r="B223" t="s">
+        <v>1102</v>
+      </c>
+      <c r="C223" t="s">
         <v>859</v>
       </c>
-      <c r="B223" t="s">
-        <v>1103</v>
-      </c>
-      <c r="C223" t="s">
+      <c r="D223" t="s">
+        <v>17</v>
+      </c>
+      <c r="E223" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F223" t="s">
         <v>860</v>
-      </c>
-      <c r="D223" t="s">
-        <v>17</v>
-      </c>
-      <c r="E223" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F223" t="s">
-        <v>861</v>
       </c>
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.15">
@@ -8291,22 +8291,22 @@
     </row>
     <row r="226" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A226" t="s">
+        <v>861</v>
+      </c>
+      <c r="B226" t="s">
         <v>862</v>
       </c>
-      <c r="B226" t="s">
+      <c r="C226" t="s">
         <v>863</v>
       </c>
-      <c r="C226" t="s">
+      <c r="D226" t="s">
         <v>864</v>
       </c>
-      <c r="D226" t="s">
+      <c r="E226" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F226" t="s">
         <v>865</v>
-      </c>
-      <c r="E226" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F226" t="s">
-        <v>866</v>
       </c>
     </row>
     <row r="227" spans="1:6" x14ac:dyDescent="0.15">
@@ -8331,10 +8331,10 @@
     </row>
     <row r="228" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A228" t="s">
+        <v>866</v>
+      </c>
+      <c r="B228" t="s">
         <v>867</v>
-      </c>
-      <c r="B228" t="s">
-        <v>868</v>
       </c>
       <c r="C228" t="s">
         <v>315</v>
@@ -8351,13 +8351,13 @@
     </row>
     <row r="229" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A229" t="s">
+        <v>880</v>
+      </c>
+      <c r="B229" t="s">
         <v>881</v>
       </c>
-      <c r="B229" t="s">
+      <c r="C229" t="s">
         <v>882</v>
-      </c>
-      <c r="C229" t="s">
-        <v>883</v>
       </c>
       <c r="D229" t="s">
         <v>49</v>
@@ -8366,18 +8366,18 @@
         <v>10</v>
       </c>
       <c r="F229" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
     </row>
     <row r="230" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A230" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="B230" t="s">
+        <v>881</v>
+      </c>
+      <c r="C230" t="s">
         <v>882</v>
-      </c>
-      <c r="C230" t="s">
-        <v>883</v>
       </c>
       <c r="D230" t="s">
         <v>49</v>
@@ -8386,15 +8386,15 @@
         <v>10</v>
       </c>
       <c r="F230" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
     </row>
     <row r="231" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A231" t="s">
+        <v>760</v>
+      </c>
+      <c r="B231" t="s">
         <v>761</v>
-      </c>
-      <c r="B231" t="s">
-        <v>762</v>
       </c>
       <c r="C231" t="s">
         <v>25</v>
@@ -8411,10 +8411,10 @@
     </row>
     <row r="232" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A232" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="B232" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="C232" t="s">
         <v>25</v>
@@ -8426,15 +8426,15 @@
         <v>10</v>
       </c>
       <c r="F232" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="233" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A233" t="s">
+        <v>763</v>
+      </c>
+      <c r="B233" t="s">
         <v>764</v>
-      </c>
-      <c r="B233" t="s">
-        <v>765</v>
       </c>
       <c r="C233" t="s">
         <v>25</v>
@@ -8446,15 +8446,15 @@
         <v>10</v>
       </c>
       <c r="F233" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="234" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A234" t="s">
+        <v>766</v>
+      </c>
+      <c r="B234" t="s">
         <v>767</v>
-      </c>
-      <c r="B234" t="s">
-        <v>768</v>
       </c>
       <c r="C234" t="s">
         <v>25</v>
@@ -8466,7 +8466,7 @@
         <v>10</v>
       </c>
       <c r="F234" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
     </row>
     <row r="235" spans="1:6" x14ac:dyDescent="0.15">
@@ -8511,16 +8511,16 @@
     </row>
     <row r="237" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A237" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B237" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="C237" t="s">
         <v>102</v>
       </c>
       <c r="D237" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="E237" t="s">
         <v>10</v>
@@ -8551,13 +8551,13 @@
     </row>
     <row r="239" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A239" t="s">
+        <v>870</v>
+      </c>
+      <c r="B239" t="s">
         <v>871</v>
       </c>
-      <c r="B239" t="s">
+      <c r="C239" t="s">
         <v>872</v>
-      </c>
-      <c r="C239" t="s">
-        <v>873</v>
       </c>
       <c r="D239" t="s">
         <v>9</v>
@@ -8566,15 +8566,15 @@
         <v>10</v>
       </c>
       <c r="F239" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="240" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A240" t="s">
+        <v>956</v>
+      </c>
+      <c r="B240" t="s">
         <v>957</v>
-      </c>
-      <c r="B240" t="s">
-        <v>958</v>
       </c>
       <c r="C240" t="s">
         <v>336</v>
@@ -8586,7 +8586,7 @@
         <v>10</v>
       </c>
       <c r="F240" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
     </row>
     <row r="241" spans="1:6" x14ac:dyDescent="0.15">
@@ -8617,7 +8617,7 @@
         <v>401</v>
       </c>
       <c r="C242" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="D242" t="s">
         <v>17</v>
@@ -8631,10 +8631,10 @@
     </row>
     <row r="243" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A243" t="s">
+        <v>769</v>
+      </c>
+      <c r="B243" t="s">
         <v>770</v>
-      </c>
-      <c r="B243" t="s">
-        <v>771</v>
       </c>
       <c r="C243" t="s">
         <v>540</v>
@@ -8691,10 +8691,10 @@
     </row>
     <row r="246" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A246" t="s">
+        <v>772</v>
+      </c>
+      <c r="B246" t="s">
         <v>773</v>
-      </c>
-      <c r="B246" t="s">
-        <v>774</v>
       </c>
       <c r="C246" t="s">
         <v>25</v>
@@ -8706,27 +8706,27 @@
         <v>10</v>
       </c>
       <c r="F246" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
     </row>
     <row r="247" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A247" t="s">
+        <v>980</v>
+      </c>
+      <c r="B247" t="s">
         <v>981</v>
       </c>
-      <c r="B247" t="s">
+      <c r="C247" t="s">
+        <v>939</v>
+      </c>
+      <c r="D247" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E247" t="s">
+        <v>10</v>
+      </c>
+      <c r="F247" t="s">
         <v>982</v>
-      </c>
-      <c r="C247" t="s">
-        <v>940</v>
-      </c>
-      <c r="D247" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E247" t="s">
-        <v>10</v>
-      </c>
-      <c r="F247" t="s">
-        <v>983</v>
       </c>
     </row>
     <row r="248" spans="1:6" x14ac:dyDescent="0.15">
@@ -8751,30 +8751,30 @@
     </row>
     <row r="249" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A249" t="s">
+        <v>885</v>
+      </c>
+      <c r="B249" t="s">
         <v>886</v>
       </c>
-      <c r="B249" t="s">
+      <c r="C249" t="s">
+        <v>1094</v>
+      </c>
+      <c r="D249" t="s">
+        <v>869</v>
+      </c>
+      <c r="E249" t="s">
+        <v>10</v>
+      </c>
+      <c r="F249" t="s">
         <v>887</v>
-      </c>
-      <c r="C249" t="s">
-        <v>1095</v>
-      </c>
-      <c r="D249" t="s">
-        <v>870</v>
-      </c>
-      <c r="E249" t="s">
-        <v>10</v>
-      </c>
-      <c r="F249" t="s">
-        <v>888</v>
       </c>
     </row>
     <row r="250" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A250" t="s">
+        <v>775</v>
+      </c>
+      <c r="B250" t="s">
         <v>776</v>
-      </c>
-      <c r="B250" t="s">
-        <v>777</v>
       </c>
       <c r="C250" t="s">
         <v>25</v>
@@ -8786,7 +8786,7 @@
         <v>10</v>
       </c>
       <c r="F250" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.15">
@@ -8811,13 +8811,13 @@
     </row>
     <row r="252" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A252" t="s">
+        <v>888</v>
+      </c>
+      <c r="B252" t="s">
         <v>889</v>
       </c>
-      <c r="B252" t="s">
+      <c r="C252" t="s">
         <v>890</v>
-      </c>
-      <c r="C252" t="s">
-        <v>891</v>
       </c>
       <c r="D252" t="s">
         <v>30</v>
@@ -8826,7 +8826,7 @@
         <v>10</v>
       </c>
       <c r="F252" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
     </row>
     <row r="253" spans="1:6" x14ac:dyDescent="0.15">
@@ -8891,10 +8891,10 @@
     </row>
     <row r="256" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A256" t="s">
+        <v>778</v>
+      </c>
+      <c r="B256" t="s">
         <v>779</v>
-      </c>
-      <c r="B256" t="s">
-        <v>780</v>
       </c>
       <c r="C256" t="s">
         <v>25</v>
@@ -8931,13 +8931,13 @@
     </row>
     <row r="258" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A258" t="s">
+        <v>780</v>
+      </c>
+      <c r="B258" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C258" t="s">
         <v>781</v>
-      </c>
-      <c r="B258" t="s">
-        <v>1098</v>
-      </c>
-      <c r="C258" t="s">
-        <v>782</v>
       </c>
       <c r="D258" t="s">
         <v>17</v>
@@ -8971,10 +8971,10 @@
     </row>
     <row r="260" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A260" t="s">
+        <v>782</v>
+      </c>
+      <c r="B260" t="s">
         <v>783</v>
-      </c>
-      <c r="B260" t="s">
-        <v>784</v>
       </c>
       <c r="C260" t="s">
         <v>25</v>
@@ -8991,10 +8991,10 @@
     </row>
     <row r="261" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A261" t="s">
+        <v>784</v>
+      </c>
+      <c r="B261" t="s">
         <v>785</v>
-      </c>
-      <c r="B261" t="s">
-        <v>786</v>
       </c>
       <c r="C261" t="s">
         <v>540</v>
@@ -9006,35 +9006,35 @@
         <v>10</v>
       </c>
       <c r="F261" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
     </row>
     <row r="262" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A262" t="s">
+        <v>787</v>
+      </c>
+      <c r="B262" t="s">
         <v>788</v>
       </c>
-      <c r="B262" t="s">
+      <c r="C262" t="s">
+        <v>1069</v>
+      </c>
+      <c r="D262" t="s">
+        <v>17</v>
+      </c>
+      <c r="E262" t="s">
+        <v>10</v>
+      </c>
+      <c r="F262" t="s">
         <v>789</v>
-      </c>
-      <c r="C262" t="s">
-        <v>1070</v>
-      </c>
-      <c r="D262" t="s">
-        <v>17</v>
-      </c>
-      <c r="E262" t="s">
-        <v>10</v>
-      </c>
-      <c r="F262" t="s">
-        <v>790</v>
       </c>
     </row>
     <row r="263" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A263" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="B263" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="C263" t="s">
         <v>25</v>
@@ -9051,10 +9051,10 @@
     </row>
     <row r="264" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A264" t="s">
+        <v>892</v>
+      </c>
+      <c r="B264" t="s">
         <v>893</v>
-      </c>
-      <c r="B264" t="s">
-        <v>894</v>
       </c>
       <c r="C264" t="s">
         <v>25</v>
@@ -9071,7 +9071,7 @@
     </row>
     <row r="265" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A265" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="B265" t="s">
         <v>39</v>
@@ -9111,33 +9111,33 @@
     </row>
     <row r="267" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A267" t="s">
+        <v>895</v>
+      </c>
+      <c r="B267" t="s">
         <v>896</v>
       </c>
-      <c r="B267" t="s">
+      <c r="C267" t="s">
         <v>897</v>
       </c>
-      <c r="C267" t="s">
+      <c r="D267" t="s">
+        <v>1072</v>
+      </c>
+      <c r="E267" t="s">
+        <v>10</v>
+      </c>
+      <c r="F267" t="s">
         <v>898</v>
-      </c>
-      <c r="D267" t="s">
-        <v>1073</v>
-      </c>
-      <c r="E267" t="s">
-        <v>10</v>
-      </c>
-      <c r="F267" t="s">
-        <v>899</v>
       </c>
     </row>
     <row r="268" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A268" t="s">
+        <v>899</v>
+      </c>
+      <c r="B268" t="s">
         <v>900</v>
       </c>
-      <c r="B268" t="s">
-        <v>901</v>
-      </c>
       <c r="C268" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="D268" t="s">
         <v>17</v>
@@ -9151,10 +9151,10 @@
     </row>
     <row r="269" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A269" t="s">
+        <v>791</v>
+      </c>
+      <c r="B269" t="s">
         <v>792</v>
-      </c>
-      <c r="B269" t="s">
-        <v>793</v>
       </c>
       <c r="C269" t="s">
         <v>540</v>
@@ -9171,30 +9171,30 @@
     </row>
     <row r="270" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A270" t="s">
+        <v>901</v>
+      </c>
+      <c r="B270" t="s">
         <v>902</v>
       </c>
-      <c r="B270" t="s">
+      <c r="C270" t="s">
+        <v>1099</v>
+      </c>
+      <c r="D270" t="s">
+        <v>864</v>
+      </c>
+      <c r="E270" t="s">
+        <v>10</v>
+      </c>
+      <c r="F270" t="s">
         <v>903</v>
-      </c>
-      <c r="C270" t="s">
-        <v>1100</v>
-      </c>
-      <c r="D270" t="s">
-        <v>865</v>
-      </c>
-      <c r="E270" t="s">
-        <v>10</v>
-      </c>
-      <c r="F270" t="s">
-        <v>904</v>
       </c>
     </row>
     <row r="271" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A271" t="s">
+        <v>793</v>
+      </c>
+      <c r="B271" t="s">
         <v>794</v>
-      </c>
-      <c r="B271" t="s">
-        <v>795</v>
       </c>
       <c r="C271" t="s">
         <v>25</v>
@@ -9206,7 +9206,7 @@
         <v>10</v>
       </c>
       <c r="F271" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="272" spans="1:6" x14ac:dyDescent="0.15">
@@ -9231,10 +9231,10 @@
     </row>
     <row r="273" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A273" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="B273" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="C273" t="s">
         <v>608</v>
@@ -9271,13 +9271,13 @@
     </row>
     <row r="275" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A275" t="s">
+        <v>906</v>
+      </c>
+      <c r="B275" t="s">
         <v>907</v>
       </c>
-      <c r="B275" t="s">
-        <v>908</v>
-      </c>
       <c r="C275" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="D275" t="s">
         <v>30</v>
@@ -9286,7 +9286,7 @@
         <v>10</v>
       </c>
       <c r="F275" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
     </row>
     <row r="276" spans="1:6" x14ac:dyDescent="0.15">
@@ -9314,7 +9314,7 @@
         <v>418</v>
       </c>
       <c r="B277" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="C277" t="s">
         <v>25</v>
@@ -9331,30 +9331,30 @@
     </row>
     <row r="278" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A278" t="s">
+        <v>909</v>
+      </c>
+      <c r="B278" t="s">
         <v>910</v>
       </c>
-      <c r="B278" t="s">
+      <c r="C278" t="s">
+        <v>1074</v>
+      </c>
+      <c r="D278" t="s">
+        <v>17</v>
+      </c>
+      <c r="E278" t="s">
+        <v>10</v>
+      </c>
+      <c r="F278" t="s">
         <v>911</v>
-      </c>
-      <c r="C278" t="s">
-        <v>1075</v>
-      </c>
-      <c r="D278" t="s">
-        <v>17</v>
-      </c>
-      <c r="E278" t="s">
-        <v>10</v>
-      </c>
-      <c r="F278" t="s">
-        <v>912</v>
       </c>
     </row>
     <row r="279" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A279" t="s">
+        <v>797</v>
+      </c>
+      <c r="B279" t="s">
         <v>798</v>
-      </c>
-      <c r="B279" t="s">
-        <v>799</v>
       </c>
       <c r="C279" t="s">
         <v>25</v>
@@ -9366,15 +9366,15 @@
         <v>10</v>
       </c>
       <c r="F279" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
     </row>
     <row r="280" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A280" t="s">
+        <v>912</v>
+      </c>
+      <c r="B280" t="s">
         <v>913</v>
-      </c>
-      <c r="B280" t="s">
-        <v>914</v>
       </c>
       <c r="C280" t="s">
         <v>204</v>
@@ -9454,7 +9454,7 @@
         <v>424</v>
       </c>
       <c r="B284" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="C284" t="s">
         <v>150</v>
@@ -9471,13 +9471,13 @@
     </row>
     <row r="285" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A285" t="s">
+        <v>914</v>
+      </c>
+      <c r="B285" t="s">
         <v>915</v>
       </c>
-      <c r="B285" t="s">
-        <v>916</v>
-      </c>
       <c r="C285" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="D285" t="s">
         <v>9</v>
@@ -9486,7 +9486,7 @@
         <v>10</v>
       </c>
       <c r="F285" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="286" spans="1:6" x14ac:dyDescent="0.15">
@@ -9511,62 +9511,62 @@
     </row>
     <row r="287" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A287" t="s">
+        <v>987</v>
+      </c>
+      <c r="B287" t="s">
         <v>988</v>
       </c>
-      <c r="B287" t="s">
+      <c r="C287" t="s">
+        <v>939</v>
+      </c>
+      <c r="D287" t="s">
+        <v>17</v>
+      </c>
+      <c r="E287" t="s">
+        <v>10</v>
+      </c>
+      <c r="F287" t="s">
         <v>989</v>
-      </c>
-      <c r="C287" t="s">
-        <v>940</v>
-      </c>
-      <c r="D287" t="s">
-        <v>17</v>
-      </c>
-      <c r="E287" t="s">
-        <v>10</v>
-      </c>
-      <c r="F287" t="s">
-        <v>990</v>
       </c>
     </row>
     <row r="288" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A288" t="s">
+        <v>990</v>
+      </c>
+      <c r="B288" t="s">
         <v>991</v>
       </c>
-      <c r="B288" t="s">
+      <c r="C288" t="s">
         <v>992</v>
       </c>
-      <c r="C288" t="s">
+      <c r="D288" t="s">
+        <v>17</v>
+      </c>
+      <c r="E288" t="s">
+        <v>10</v>
+      </c>
+      <c r="F288" t="s">
         <v>993</v>
-      </c>
-      <c r="D288" t="s">
-        <v>17</v>
-      </c>
-      <c r="E288" t="s">
-        <v>10</v>
-      </c>
-      <c r="F288" t="s">
-        <v>994</v>
       </c>
     </row>
     <row r="289" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A289" t="s">
+        <v>959</v>
+      </c>
+      <c r="B289" t="s">
         <v>960</v>
       </c>
-      <c r="B289" t="s">
+      <c r="C289" t="s">
+        <v>939</v>
+      </c>
+      <c r="D289" t="s">
+        <v>17</v>
+      </c>
+      <c r="E289" t="s">
+        <v>10</v>
+      </c>
+      <c r="F289" t="s">
         <v>961</v>
-      </c>
-      <c r="C289" t="s">
-        <v>940</v>
-      </c>
-      <c r="D289" t="s">
-        <v>17</v>
-      </c>
-      <c r="E289" t="s">
-        <v>10</v>
-      </c>
-      <c r="F289" t="s">
-        <v>962</v>
       </c>
     </row>
     <row r="290" spans="1:6" x14ac:dyDescent="0.15">
@@ -9631,10 +9631,10 @@
     </row>
     <row r="293" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A293" t="s">
+        <v>800</v>
+      </c>
+      <c r="B293" t="s">
         <v>801</v>
-      </c>
-      <c r="B293" t="s">
-        <v>802</v>
       </c>
       <c r="C293" t="s">
         <v>25</v>
@@ -9714,7 +9714,7 @@
         <v>436</v>
       </c>
       <c r="B297" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="C297" t="s">
         <v>136</v>
@@ -9731,22 +9731,22 @@
     </row>
     <row r="298" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A298" t="s">
+        <v>918</v>
+      </c>
+      <c r="B298" t="s">
         <v>919</v>
       </c>
-      <c r="B298" t="s">
+      <c r="C298" t="s">
         <v>920</v>
       </c>
-      <c r="C298" t="s">
+      <c r="D298" t="s">
+        <v>17</v>
+      </c>
+      <c r="E298" t="s">
+        <v>10</v>
+      </c>
+      <c r="F298" t="s">
         <v>921</v>
-      </c>
-      <c r="D298" t="s">
-        <v>17</v>
-      </c>
-      <c r="E298" t="s">
-        <v>10</v>
-      </c>
-      <c r="F298" t="s">
-        <v>922</v>
       </c>
     </row>
     <row r="299" spans="1:6" x14ac:dyDescent="0.15">
@@ -9771,13 +9771,13 @@
     </row>
     <row r="300" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A300" t="s">
+        <v>922</v>
+      </c>
+      <c r="B300" t="s">
         <v>923</v>
       </c>
-      <c r="B300" t="s">
+      <c r="C300" t="s">
         <v>924</v>
-      </c>
-      <c r="C300" t="s">
-        <v>925</v>
       </c>
       <c r="D300" t="s">
         <v>17</v>
@@ -9791,30 +9791,30 @@
     </row>
     <row r="301" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A301" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B301" t="s">
+        <v>925</v>
+      </c>
+      <c r="C301" t="s">
         <v>1058</v>
       </c>
-      <c r="B301" t="s">
+      <c r="D301" t="s">
+        <v>17</v>
+      </c>
+      <c r="E301" t="s">
+        <v>10</v>
+      </c>
+      <c r="F301" t="s">
         <v>926</v>
-      </c>
-      <c r="C301" t="s">
-        <v>1059</v>
-      </c>
-      <c r="D301" t="s">
-        <v>17</v>
-      </c>
-      <c r="E301" t="s">
-        <v>10</v>
-      </c>
-      <c r="F301" t="s">
-        <v>927</v>
       </c>
     </row>
     <row r="302" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A302" t="s">
+        <v>802</v>
+      </c>
+      <c r="B302" t="s">
         <v>803</v>
-      </c>
-      <c r="B302" t="s">
-        <v>804</v>
       </c>
       <c r="C302" t="s">
         <v>545</v>
@@ -9854,7 +9854,7 @@
         <v>642</v>
       </c>
       <c r="B304" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="C304" t="s">
         <v>25</v>
@@ -9891,30 +9891,30 @@
     </row>
     <row r="306" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A306" t="s">
+        <v>962</v>
+      </c>
+      <c r="B306" t="s">
         <v>963</v>
       </c>
-      <c r="B306" t="s">
+      <c r="C306" t="s">
+        <v>939</v>
+      </c>
+      <c r="D306" t="s">
+        <v>17</v>
+      </c>
+      <c r="E306" t="s">
+        <v>10</v>
+      </c>
+      <c r="F306" t="s">
         <v>964</v>
-      </c>
-      <c r="C306" t="s">
-        <v>940</v>
-      </c>
-      <c r="D306" t="s">
-        <v>17</v>
-      </c>
-      <c r="E306" t="s">
-        <v>10</v>
-      </c>
-      <c r="F306" t="s">
-        <v>965</v>
       </c>
     </row>
     <row r="307" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A307" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B307" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="C307" t="s">
         <v>25</v>
@@ -9926,7 +9926,7 @@
         <v>10</v>
       </c>
       <c r="F307" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
     </row>
     <row r="308" spans="1:6" x14ac:dyDescent="0.15">
@@ -9971,10 +9971,10 @@
     </row>
     <row r="310" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A310" t="s">
+        <v>927</v>
+      </c>
+      <c r="B310" t="s">
         <v>928</v>
-      </c>
-      <c r="B310" t="s">
-        <v>929</v>
       </c>
       <c r="C310" t="s">
         <v>310</v>
@@ -9986,15 +9986,15 @@
         <v>10</v>
       </c>
       <c r="F310" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="311" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A311" t="s">
+        <v>930</v>
+      </c>
+      <c r="B311" t="s">
         <v>931</v>
-      </c>
-      <c r="B311" t="s">
-        <v>932</v>
       </c>
       <c r="C311" t="s">
         <v>180</v>
@@ -10051,13 +10051,13 @@
     </row>
     <row r="314" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A314" t="s">
+        <v>805</v>
+      </c>
+      <c r="B314" t="s">
         <v>806</v>
       </c>
-      <c r="B314" t="s">
+      <c r="C314" t="s">
         <v>807</v>
-      </c>
-      <c r="C314" t="s">
-        <v>808</v>
       </c>
       <c r="D314" t="s">
         <v>49</v>
@@ -10071,10 +10071,10 @@
     </row>
     <row r="315" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A315" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="B315" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="C315" t="s">
         <v>25</v>
@@ -10086,7 +10086,7 @@
         <v>10</v>
       </c>
       <c r="F315" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
     </row>
     <row r="316" spans="1:6" x14ac:dyDescent="0.15">
@@ -10094,7 +10094,7 @@
         <v>451</v>
       </c>
       <c r="B316" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="C316" t="s">
         <v>158</v>
@@ -10137,7 +10137,7 @@
         <v>455</v>
       </c>
       <c r="C318" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="D318" t="s">
         <v>17</v>
@@ -10154,7 +10154,7 @@
         <v>457</v>
       </c>
       <c r="B319" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="C319" t="s">
         <v>152</v>
@@ -10191,10 +10191,10 @@
     </row>
     <row r="321" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A321" t="s">
+        <v>932</v>
+      </c>
+      <c r="B321" t="s">
         <v>933</v>
-      </c>
-      <c r="B321" t="s">
-        <v>934</v>
       </c>
       <c r="C321" t="s">
         <v>25</v>
@@ -10211,10 +10211,10 @@
     </row>
     <row r="322" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A322" t="s">
+        <v>904</v>
+      </c>
+      <c r="B322" t="s">
         <v>905</v>
-      </c>
-      <c r="B322" t="s">
-        <v>906</v>
       </c>
       <c r="C322" t="s">
         <v>336</v>
@@ -10231,10 +10231,10 @@
     </row>
     <row r="323" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A323" t="s">
+        <v>998</v>
+      </c>
+      <c r="B323" t="s">
         <v>999</v>
-      </c>
-      <c r="B323" t="s">
-        <v>1000</v>
       </c>
       <c r="C323" t="s">
         <v>136</v>
@@ -10246,15 +10246,15 @@
         <v>10</v>
       </c>
       <c r="F323" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="324" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A324" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B324" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="C324" t="s">
         <v>136</v>
@@ -10266,15 +10266,15 @@
         <v>10</v>
       </c>
       <c r="F324" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="325" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A325" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B325" t="s">
         <v>1003</v>
-      </c>
-      <c r="B325" t="s">
-        <v>1004</v>
       </c>
       <c r="C325" t="s">
         <v>25</v>
@@ -10286,7 +10286,7 @@
         <v>10</v>
       </c>
       <c r="F325" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="326" spans="1:6" x14ac:dyDescent="0.15">
@@ -10294,7 +10294,7 @@
         <v>460</v>
       </c>
       <c r="B326" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="C326" t="s">
         <v>158</v>
@@ -10311,10 +10311,10 @@
     </row>
     <row r="327" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A327" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B327" t="s">
         <v>1006</v>
-      </c>
-      <c r="B327" t="s">
-        <v>1007</v>
       </c>
       <c r="C327" t="s">
         <v>136</v>
@@ -10326,7 +10326,7 @@
         <v>10</v>
       </c>
       <c r="F327" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="328" spans="1:6" x14ac:dyDescent="0.15">
@@ -10351,30 +10351,30 @@
     </row>
     <row r="329" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A329" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B329" t="s">
         <v>1009</v>
       </c>
-      <c r="B329" t="s">
+      <c r="C329" t="s">
         <v>1010</v>
       </c>
-      <c r="C329" t="s">
+      <c r="D329" t="s">
         <v>1011</v>
       </c>
-      <c r="D329" t="s">
+      <c r="E329" t="s">
+        <v>10</v>
+      </c>
+      <c r="F329" t="s">
         <v>1012</v>
-      </c>
-      <c r="E329" t="s">
-        <v>10</v>
-      </c>
-      <c r="F329" t="s">
-        <v>1013</v>
       </c>
     </row>
     <row r="330" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A330" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="B330" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="C330" t="s">
         <v>540</v>
@@ -10431,13 +10431,13 @@
     </row>
     <row r="333" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A333" t="s">
+        <v>996</v>
+      </c>
+      <c r="B333" t="s">
         <v>997</v>
       </c>
-      <c r="B333" t="s">
-        <v>998</v>
-      </c>
       <c r="C333" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="D333" t="s">
         <v>17</v>
@@ -10446,7 +10446,7 @@
         <v>10</v>
       </c>
       <c r="F333" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="334" spans="1:6" x14ac:dyDescent="0.15">
@@ -10457,7 +10457,7 @@
         <v>471</v>
       </c>
       <c r="C334" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="D334" t="s">
         <v>17</v>
@@ -10471,10 +10471,10 @@
     </row>
     <row r="335" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A335" t="s">
+        <v>811</v>
+      </c>
+      <c r="B335" t="s">
         <v>812</v>
-      </c>
-      <c r="B335" t="s">
-        <v>813</v>
       </c>
       <c r="C335" t="s">
         <v>25</v>
@@ -10531,10 +10531,10 @@
     </row>
     <row r="338" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A338" t="s">
+        <v>714</v>
+      </c>
+      <c r="B338" t="s">
         <v>715</v>
-      </c>
-      <c r="B338" t="s">
-        <v>716</v>
       </c>
       <c r="C338" t="s">
         <v>608</v>
@@ -10551,33 +10551,33 @@
     </row>
     <row r="339" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A339" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B339" t="s">
         <v>1014</v>
       </c>
-      <c r="B339" t="s">
-        <v>1015</v>
-      </c>
       <c r="C339" t="s">
+        <v>916</v>
+      </c>
+      <c r="D339" t="s">
+        <v>17</v>
+      </c>
+      <c r="E339" t="s">
+        <v>10</v>
+      </c>
+      <c r="F339" t="s">
         <v>917</v>
-      </c>
-      <c r="D339" t="s">
-        <v>17</v>
-      </c>
-      <c r="E339" t="s">
-        <v>10</v>
-      </c>
-      <c r="F339" t="s">
-        <v>918</v>
       </c>
     </row>
     <row r="340" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A340" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B340" t="s">
         <v>1016</v>
       </c>
-      <c r="B340" t="s">
+      <c r="C340" t="s">
         <v>1017</v>
-      </c>
-      <c r="C340" t="s">
-        <v>1018</v>
       </c>
       <c r="D340" t="s">
         <v>143</v>
@@ -10586,15 +10586,15 @@
         <v>10</v>
       </c>
       <c r="F340" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="341" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A341" t="s">
+        <v>813</v>
+      </c>
+      <c r="B341" t="s">
         <v>814</v>
-      </c>
-      <c r="B341" t="s">
-        <v>815</v>
       </c>
       <c r="C341" t="s">
         <v>540</v>
@@ -10611,22 +10611,22 @@
     </row>
     <row r="342" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A342" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B342" t="s">
         <v>1019</v>
       </c>
-      <c r="B342" t="s">
+      <c r="C342" t="s">
+        <v>1103</v>
+      </c>
+      <c r="D342" t="s">
         <v>1020</v>
       </c>
-      <c r="C342" t="s">
-        <v>1104</v>
-      </c>
-      <c r="D342" t="s">
+      <c r="E342" t="s">
+        <v>10</v>
+      </c>
+      <c r="F342" t="s">
         <v>1021</v>
-      </c>
-      <c r="E342" t="s">
-        <v>10</v>
-      </c>
-      <c r="F342" t="s">
-        <v>1022</v>
       </c>
     </row>
     <row r="343" spans="1:6" x14ac:dyDescent="0.15">
@@ -10651,13 +10651,13 @@
     </row>
     <row r="344" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A344" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B344" t="s">
         <v>1023</v>
       </c>
-      <c r="B344" t="s">
-        <v>1024</v>
-      </c>
       <c r="C344" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="D344" t="s">
         <v>9</v>
@@ -10666,7 +10666,7 @@
         <v>10</v>
       </c>
       <c r="F344" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="345" spans="1:6" x14ac:dyDescent="0.15">
@@ -10691,13 +10691,13 @@
     </row>
     <row r="346" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A346" t="s">
+        <v>965</v>
+      </c>
+      <c r="B346" t="s">
         <v>966</v>
       </c>
-      <c r="B346" t="s">
-        <v>967</v>
-      </c>
       <c r="C346" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="D346" s="1" t="s">
         <v>17</v>
@@ -10706,7 +10706,7 @@
         <v>10</v>
       </c>
       <c r="F346" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="347" spans="1:6" x14ac:dyDescent="0.15">
@@ -10751,10 +10751,10 @@
     </row>
     <row r="349" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A349" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="B349" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="C349" t="s">
         <v>25</v>
@@ -10766,15 +10766,15 @@
         <v>10</v>
       </c>
       <c r="F349" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="350" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A350" t="s">
+        <v>815</v>
+      </c>
+      <c r="B350" t="s">
         <v>816</v>
-      </c>
-      <c r="B350" t="s">
-        <v>817</v>
       </c>
       <c r="C350" t="s">
         <v>25</v>
@@ -10786,7 +10786,7 @@
         <v>10</v>
       </c>
       <c r="F350" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
     </row>
     <row r="351" spans="1:6" x14ac:dyDescent="0.15">
@@ -10811,10 +10811,10 @@
     </row>
     <row r="352" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A352" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="B352" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="C352" t="s">
         <v>25</v>
@@ -10831,22 +10831,22 @@
     </row>
     <row r="353" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A353" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B353" t="s">
         <v>1026</v>
       </c>
-      <c r="B353" t="s">
+      <c r="C353" t="s">
         <v>1027</v>
       </c>
-      <c r="C353" t="s">
+      <c r="D353" t="s">
+        <v>17</v>
+      </c>
+      <c r="E353" t="s">
+        <v>10</v>
+      </c>
+      <c r="F353" t="s">
         <v>1028</v>
-      </c>
-      <c r="D353" t="s">
-        <v>17</v>
-      </c>
-      <c r="E353" t="s">
-        <v>10</v>
-      </c>
-      <c r="F353" t="s">
-        <v>1029</v>
       </c>
     </row>
     <row r="354" spans="1:6" x14ac:dyDescent="0.15">
@@ -10877,7 +10877,7 @@
         <v>648</v>
       </c>
       <c r="C355" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="D355" t="s">
         <v>17</v>
@@ -10931,10 +10931,10 @@
     </row>
     <row r="358" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A358" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="B358" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="C358" t="s">
         <v>25</v>
@@ -10946,7 +10946,7 @@
         <v>10</v>
       </c>
       <c r="F358" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="359" spans="1:6" x14ac:dyDescent="0.15">
@@ -10971,10 +10971,10 @@
     </row>
     <row r="360" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A360" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B360" t="s">
         <v>1033</v>
-      </c>
-      <c r="B360" t="s">
-        <v>1034</v>
       </c>
       <c r="C360" t="s">
         <v>150</v>
@@ -10991,13 +10991,13 @@
     </row>
     <row r="361" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A361" t="s">
+        <v>1034</v>
+      </c>
+      <c r="B361" t="s">
         <v>1035</v>
       </c>
-      <c r="B361" t="s">
-        <v>1036</v>
-      </c>
       <c r="C361" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="D361" t="s">
         <v>17</v>
@@ -11011,30 +11011,30 @@
     </row>
     <row r="362" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A362" t="s">
+        <v>967</v>
+      </c>
+      <c r="B362" t="s">
         <v>968</v>
       </c>
-      <c r="B362" t="s">
+      <c r="C362" t="s">
+        <v>939</v>
+      </c>
+      <c r="D362" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E362" t="s">
+        <v>10</v>
+      </c>
+      <c r="F362" t="s">
         <v>969</v>
-      </c>
-      <c r="C362" t="s">
-        <v>940</v>
-      </c>
-      <c r="D362" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E362" t="s">
-        <v>10</v>
-      </c>
-      <c r="F362" t="s">
-        <v>970</v>
       </c>
     </row>
     <row r="363" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A363" t="s">
+        <v>817</v>
+      </c>
+      <c r="B363" t="s">
         <v>818</v>
-      </c>
-      <c r="B363" t="s">
-        <v>819</v>
       </c>
       <c r="C363" t="s">
         <v>25</v>
@@ -11051,10 +11051,10 @@
     </row>
     <row r="364" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A364" t="s">
+        <v>819</v>
+      </c>
+      <c r="B364" t="s">
         <v>820</v>
-      </c>
-      <c r="B364" t="s">
-        <v>821</v>
       </c>
       <c r="C364" t="s">
         <v>552</v>
@@ -11091,10 +11091,10 @@
     </row>
     <row r="366" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A366" t="s">
+        <v>821</v>
+      </c>
+      <c r="B366" t="s">
         <v>822</v>
-      </c>
-      <c r="B366" t="s">
-        <v>823</v>
       </c>
       <c r="C366" t="s">
         <v>545</v>
@@ -11120,7 +11120,7 @@
         <v>489</v>
       </c>
       <c r="D367" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="E367" t="s">
         <v>10</v>
@@ -11171,22 +11171,22 @@
     </row>
     <row r="370" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A370" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B370" t="s">
         <v>1037</v>
       </c>
-      <c r="B370" t="s">
+      <c r="C370" t="s">
         <v>1038</v>
       </c>
-      <c r="C370" t="s">
+      <c r="D370" t="s">
+        <v>17</v>
+      </c>
+      <c r="E370" t="s">
+        <v>10</v>
+      </c>
+      <c r="F370" t="s">
         <v>1039</v>
-      </c>
-      <c r="D370" t="s">
-        <v>17</v>
-      </c>
-      <c r="E370" t="s">
-        <v>10</v>
-      </c>
-      <c r="F370" t="s">
-        <v>1040</v>
       </c>
     </row>
     <row r="371" spans="1:6" x14ac:dyDescent="0.15">
@@ -11217,7 +11217,7 @@
         <v>659</v>
       </c>
       <c r="C372" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="D372" t="s">
         <v>17</v>
@@ -11231,22 +11231,22 @@
     </row>
     <row r="373" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A373" t="s">
+        <v>970</v>
+      </c>
+      <c r="B373" t="s">
         <v>971</v>
       </c>
-      <c r="B373" t="s">
+      <c r="C373" t="s">
         <v>972</v>
       </c>
-      <c r="C373" t="s">
+      <c r="D373" t="s">
+        <v>17</v>
+      </c>
+      <c r="E373" t="s">
+        <v>10</v>
+      </c>
+      <c r="F373" t="s">
         <v>973</v>
-      </c>
-      <c r="D373" t="s">
-        <v>17</v>
-      </c>
-      <c r="E373" t="s">
-        <v>10</v>
-      </c>
-      <c r="F373" t="s">
-        <v>974</v>
       </c>
     </row>
     <row r="374" spans="1:6" x14ac:dyDescent="0.15">
@@ -11271,10 +11271,10 @@
     </row>
     <row r="375" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A375" t="s">
+        <v>823</v>
+      </c>
+      <c r="B375" t="s">
         <v>824</v>
-      </c>
-      <c r="B375" t="s">
-        <v>825</v>
       </c>
       <c r="C375" t="s">
         <v>25</v>
@@ -11286,7 +11286,7 @@
         <v>10</v>
       </c>
       <c r="F375" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="376" spans="1:6" x14ac:dyDescent="0.15">
@@ -11311,10 +11311,10 @@
     </row>
     <row r="377" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A377" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B377" t="s">
         <v>1041</v>
-      </c>
-      <c r="B377" t="s">
-        <v>1042</v>
       </c>
       <c r="C377" t="s">
         <v>25</v>
@@ -11351,10 +11351,10 @@
     </row>
     <row r="379" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A379" t="s">
+        <v>826</v>
+      </c>
+      <c r="B379" t="s">
         <v>827</v>
-      </c>
-      <c r="B379" t="s">
-        <v>828</v>
       </c>
       <c r="C379" t="s">
         <v>558</v>
@@ -11391,10 +11391,10 @@
     </row>
     <row r="381" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A381" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B381" t="s">
         <v>1043</v>
-      </c>
-      <c r="B381" t="s">
-        <v>1044</v>
       </c>
       <c r="C381" t="s">
         <v>545</v>
@@ -11411,22 +11411,22 @@
     </row>
     <row r="382" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A382" t="s">
+        <v>828</v>
+      </c>
+      <c r="B382" t="s">
         <v>829</v>
       </c>
-      <c r="B382" t="s">
+      <c r="C382" t="s">
         <v>830</v>
       </c>
-      <c r="C382" t="s">
+      <c r="D382" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E382" t="s">
+        <v>10</v>
+      </c>
+      <c r="F382" t="s">
         <v>831</v>
-      </c>
-      <c r="D382" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E382" t="s">
-        <v>10</v>
-      </c>
-      <c r="F382" t="s">
-        <v>832</v>
       </c>
     </row>
     <row r="383" spans="1:6" x14ac:dyDescent="0.15">
@@ -11434,7 +11434,7 @@
         <v>496</v>
       </c>
       <c r="B383" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="C383" t="s">
         <v>48</v>
@@ -11471,10 +11471,10 @@
     </row>
     <row r="385" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A385" t="s">
+        <v>832</v>
+      </c>
+      <c r="B385" t="s">
         <v>833</v>
-      </c>
-      <c r="B385" t="s">
-        <v>834</v>
       </c>
       <c r="C385" t="s">
         <v>552</v>
@@ -11497,7 +11497,7 @@
         <v>670</v>
       </c>
       <c r="C386" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="D386" t="s">
         <v>17</v>
@@ -11511,13 +11511,13 @@
     </row>
     <row r="387" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A387" t="s">
+        <v>994</v>
+      </c>
+      <c r="B387" t="s">
         <v>995</v>
       </c>
-      <c r="B387" t="s">
-        <v>996</v>
-      </c>
       <c r="C387" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="D387" t="s">
         <v>17</v>
@@ -11526,7 +11526,7 @@
         <v>10</v>
       </c>
       <c r="F387" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="388" spans="1:6" x14ac:dyDescent="0.15">
@@ -11551,10 +11551,10 @@
     </row>
     <row r="389" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A389" t="s">
+        <v>834</v>
+      </c>
+      <c r="B389" t="s">
         <v>835</v>
-      </c>
-      <c r="B389" t="s">
-        <v>836</v>
       </c>
       <c r="C389" t="s">
         <v>552</v>
@@ -11566,15 +11566,15 @@
         <v>10</v>
       </c>
       <c r="F389" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="390" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A390" t="s">
+        <v>837</v>
+      </c>
+      <c r="B390" t="s">
         <v>838</v>
-      </c>
-      <c r="B390" t="s">
-        <v>839</v>
       </c>
       <c r="C390" t="s">
         <v>552</v>
@@ -11591,42 +11591,42 @@
     </row>
     <row r="391" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A391" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B391" t="s">
         <v>1045</v>
       </c>
-      <c r="B391" t="s">
+      <c r="C391" t="s">
+        <v>1115</v>
+      </c>
+      <c r="D391" t="s">
+        <v>17</v>
+      </c>
+      <c r="E391" t="s">
+        <v>10</v>
+      </c>
+      <c r="F391" t="s">
         <v>1046</v>
-      </c>
-      <c r="C391" t="s">
-        <v>1116</v>
-      </c>
-      <c r="D391" t="s">
-        <v>17</v>
-      </c>
-      <c r="E391" t="s">
-        <v>10</v>
-      </c>
-      <c r="F391" t="s">
-        <v>1047</v>
       </c>
     </row>
     <row r="392" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A392" t="s">
+        <v>1047</v>
+      </c>
+      <c r="B392" t="s">
         <v>1048</v>
       </c>
-      <c r="B392" t="s">
+      <c r="C392" t="s">
+        <v>1086</v>
+      </c>
+      <c r="D392" t="s">
         <v>1049</v>
       </c>
-      <c r="C392" t="s">
-        <v>1087</v>
-      </c>
-      <c r="D392" t="s">
+      <c r="E392" t="s">
+        <v>10</v>
+      </c>
+      <c r="F392" t="s">
         <v>1050</v>
-      </c>
-      <c r="E392" t="s">
-        <v>10</v>
-      </c>
-      <c r="F392" t="s">
-        <v>1051</v>
       </c>
     </row>
     <row r="393" spans="1:6" x14ac:dyDescent="0.15">

</xml_diff>